<commit_message>
Updated the BOM Added part placement files
</commit_message>
<xml_diff>
--- a/Hardware/final/ZIPPY PROTO BADGE BOM.xlsx
+++ b/Hardware/final/ZIPPY PROTO BADGE BOM.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="28623"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="28925"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\hamster\Documents\Development\Badges\dczia\zippy-badge\proto\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\hamster\Documents\Development\Badges\dczia\zippy-badge\Hardware\final\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8681E254-8B07-4DD6-9706-63FEAE1E5BB4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1BFBA32A-244F-43A5-93C1-A11A8DA1111D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="11330" yWindow="960" windowWidth="25300" windowHeight="17810" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="8830" yWindow="3110" windowWidth="25670" windowHeight="16210" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="BOM" sheetId="1" r:id="rId1"/>
@@ -33,7 +33,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="145" uniqueCount="108">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="176" uniqueCount="132">
   <si>
     <t>Part Number</t>
   </si>
@@ -98,9 +98,6 @@
     <t>Qty</t>
   </si>
   <si>
-    <t>C1,C2,C3,C4,C5,C6,C7,C12,C15,C16,C17,C18,C19,C20</t>
-  </si>
-  <si>
     <t>~</t>
   </si>
   <si>
@@ -110,12 +107,6 @@
     <t>C11,C13</t>
   </si>
   <si>
-    <t>27pF</t>
-  </si>
-  <si>
-    <t>D1</t>
-  </si>
-  <si>
     <t>D_Schottky</t>
   </si>
   <si>
@@ -356,7 +347,88 @@
     <t>https://www.aliexpress.us/item/2251832628463811.html?spm=a2g0o.order_list.order_list_main.10.75b61802s7r8Fm&amp;gatewayAdapt=glo2usa</t>
   </si>
   <si>
-    <t>Total</t>
+    <t>C1, C2, C3, C4, C5, C6, C7, C12, C15, C16, C17, C18, C19, C20, C21, C22</t>
+  </si>
+  <si>
+    <t>15pF</t>
+  </si>
+  <si>
+    <t>D1, D45</t>
+  </si>
+  <si>
+    <t>J3</t>
+  </si>
+  <si>
+    <t>1x8 Pin Header</t>
+  </si>
+  <si>
+    <t>DNS</t>
+  </si>
+  <si>
+    <t>J4</t>
+  </si>
+  <si>
+    <t>1x10 Pin Header</t>
+  </si>
+  <si>
+    <t>SW3</t>
+  </si>
+  <si>
+    <t>SKRHABE010</t>
+  </si>
+  <si>
+    <t>D-Pad</t>
+  </si>
+  <si>
+    <t>688-SKRHAAE010</t>
+  </si>
+  <si>
+    <t>https://www.mouser.com/datasheet/2/15/SKRH-1370966.pdf</t>
+  </si>
+  <si>
+    <t>TP5, TP6</t>
+  </si>
+  <si>
+    <t>Spare</t>
+  </si>
+  <si>
+    <t>U4</t>
+  </si>
+  <si>
+    <t>GSDA213</t>
+  </si>
+  <si>
+    <t>Kionix_LGA-12_2x2mm_P0.5mm_LayoutBorder2x4y</t>
+  </si>
+  <si>
+    <t>Digikey</t>
+  </si>
+  <si>
+    <t>4786-GSDA213TR-ND</t>
+  </si>
+  <si>
+    <t>https://goodarksemi.com/docs/datasheets/mems/GSDA213_SDS.pdf</t>
+  </si>
+  <si>
+    <t>MK1</t>
+  </si>
+  <si>
+    <t>ICS-43434</t>
+  </si>
+  <si>
+    <t>InvenSense_ICS-43434-6_3.5x2.65mm</t>
+  </si>
+  <si>
+    <t>Total Parts</t>
+  </si>
+  <si>
+    <t>PCB</t>
+  </si>
+  <si>
+    <t>Batteries</t>
+  </si>
+  <si>
+    <t>Amazon</t>
   </si>
 </sst>
 </file>
@@ -438,7 +510,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="21">
+  <cellXfs count="19">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
@@ -450,18 +522,16 @@
     <xf numFmtId="49" fontId="3" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
     <xf numFmtId="49" fontId="4" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
     <xf numFmtId="49" fontId="7" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="1" applyNumberFormat="1"/>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
     <xf numFmtId="49" fontId="6" fillId="0" borderId="0" xfId="1" applyNumberFormat="1"/>
@@ -752,10 +822,10 @@
   <sheetPr>
     <outlinePr summaryBelow="0" summaryRight="0"/>
   </sheetPr>
-  <dimension ref="A1:O981"/>
+  <dimension ref="A1:O988"/>
   <sheetFormatPr defaultColWidth="14.453125" defaultRowHeight="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="12.08984375" customWidth="1"/>
+    <col min="1" max="1" width="22.36328125" customWidth="1"/>
     <col min="2" max="2" width="17.54296875" customWidth="1"/>
     <col min="3" max="3" width="35.54296875" style="5" customWidth="1"/>
     <col min="4" max="4" width="21.1796875" customWidth="1"/>
@@ -772,53 +842,53 @@
     <col min="16" max="16" width="12.90625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:14" s="18" customFormat="1" ht="35.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="16" t="s">
+    <row r="1" spans="1:14" s="16" customFormat="1" ht="35.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A1" s="14" t="s">
         <v>16</v>
       </c>
-      <c r="B1" s="17" t="s">
+      <c r="B1" s="15" t="s">
         <v>17</v>
       </c>
-      <c r="C1" s="20" t="s">
+      <c r="C1" s="18" t="s">
         <v>18</v>
       </c>
-      <c r="D1" s="17" t="s">
-        <v>0</v>
-      </c>
-      <c r="E1" s="17" t="s">
+      <c r="D1" s="15" t="s">
+        <v>0</v>
+      </c>
+      <c r="E1" s="15" t="s">
+        <v>73</v>
+      </c>
+      <c r="F1" s="15" t="s">
+        <v>74</v>
+      </c>
+      <c r="G1" s="16" t="s">
+        <v>19</v>
+      </c>
+      <c r="H1" s="15" t="s">
+        <v>20</v>
+      </c>
+      <c r="I1" s="15" t="s">
+        <v>71</v>
+      </c>
+      <c r="J1" s="15" t="s">
+        <v>72</v>
+      </c>
+      <c r="K1" s="15" t="s">
+        <v>75</v>
+      </c>
+      <c r="L1" s="15" t="s">
         <v>76</v>
       </c>
-      <c r="F1" s="17" t="s">
-        <v>77</v>
-      </c>
-      <c r="G1" s="18" t="s">
-        <v>19</v>
-      </c>
-      <c r="H1" s="17" t="s">
-        <v>20</v>
-      </c>
-      <c r="I1" s="17" t="s">
-        <v>74</v>
-      </c>
-      <c r="J1" s="17" t="s">
-        <v>75</v>
-      </c>
-      <c r="K1" s="17" t="s">
-        <v>78</v>
-      </c>
-      <c r="L1" s="17" t="s">
-        <v>79</v>
-      </c>
-      <c r="M1" s="17" t="s">
+      <c r="M1" s="15" t="s">
         <v>1</v>
       </c>
-      <c r="N1" s="17" t="s">
-        <v>100</v>
+      <c r="N1" s="15" t="s">
+        <v>97</v>
       </c>
     </row>
     <row r="2" spans="1:14" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A2" s="1" t="s">
-        <v>21</v>
+        <v>104</v>
       </c>
       <c r="B2" t="s">
         <v>3</v>
@@ -827,65 +897,64 @@
         <v>9</v>
       </c>
       <c r="G2" s="5" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="H2">
         <v>14</v>
       </c>
-      <c r="I2" s="11">
+      <c r="I2">
         <v>4.0000000000000001E-3</v>
       </c>
-      <c r="J2" s="11">
+      <c r="J2">
         <f>H2*I2</f>
         <v>5.6000000000000001E-2</v>
       </c>
-      <c r="K2" s="11">
-        <v>0</v>
-      </c>
-      <c r="L2" s="11">
-        <v>0</v>
-      </c>
-      <c r="M2" s="11">
+      <c r="K2">
+        <v>0</v>
+      </c>
+      <c r="L2">
+        <v>0</v>
+      </c>
+      <c r="M2">
         <v>5000</v>
       </c>
     </row>
     <row r="3" spans="1:14" s="1" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A3" s="1" t="s">
-        <v>102</v>
+        <v>99</v>
       </c>
       <c r="B3" s="1" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="C3" s="8" t="s">
         <v>9</v>
       </c>
       <c r="G3" s="6" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="H3" s="1">
-        <v>2</v>
-      </c>
-      <c r="I3" s="12">
+        <v>4</v>
+      </c>
+      <c r="I3" s="1">
         <v>4.0000000000000001E-3</v>
       </c>
-      <c r="J3" s="11">
-        <f t="shared" ref="J3:J36" si="0">H3*I3</f>
-        <v>8.0000000000000002E-3</v>
-      </c>
-      <c r="K3" s="12">
-        <v>0</v>
-      </c>
-      <c r="L3" s="12">
+      <c r="J3">
+        <f t="shared" ref="J3:J44" si="0">H3*I3</f>
+        <v>1.6E-2</v>
+      </c>
+      <c r="K3" s="1">
+        <v>0</v>
+      </c>
+      <c r="L3" s="1">
         <v>4000</v>
       </c>
-      <c r="M3" s="12"/>
     </row>
     <row r="4" spans="1:14" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A4" s="1" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="B4" t="s">
-        <v>25</v>
+        <v>105</v>
       </c>
       <c r="C4" s="8" t="s">
         <v>9</v>
@@ -894,25 +963,24 @@
       <c r="E4" s="3"/>
       <c r="F4" s="3"/>
       <c r="G4" s="5" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="H4" s="3">
         <v>2</v>
       </c>
-      <c r="I4" s="11">
+      <c r="I4">
         <v>4.0000000000000001E-3</v>
       </c>
-      <c r="J4" s="11">
+      <c r="J4">
         <f t="shared" si="0"/>
         <v>8.0000000000000002E-3</v>
       </c>
-      <c r="K4" s="11">
-        <v>0</v>
-      </c>
-      <c r="L4" s="11">
+      <c r="K4">
+        <v>0</v>
+      </c>
+      <c r="L4">
         <v>4000</v>
       </c>
-      <c r="M4" s="11"/>
     </row>
     <row r="5" spans="1:14" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A5" s="1"/>
@@ -921,927 +989,1020 @@
       <c r="E5" s="3"/>
       <c r="F5" s="3"/>
       <c r="H5" s="3"/>
-      <c r="I5" s="11"/>
-      <c r="J5" s="11"/>
-      <c r="K5" s="11"/>
-      <c r="L5" s="11"/>
-      <c r="M5" s="11"/>
+      <c r="J5"/>
     </row>
     <row r="6" spans="1:14" s="1" customFormat="1" ht="12.5" x14ac:dyDescent="0.25">
       <c r="A6" s="1" t="s">
-        <v>26</v>
+        <v>106</v>
       </c>
       <c r="B6" s="1" t="s">
-        <v>27</v>
+        <v>24</v>
       </c>
       <c r="C6" s="6" t="s">
-        <v>28</v>
+        <v>25</v>
       </c>
       <c r="G6" s="6" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="H6" s="1">
-        <v>1</v>
-      </c>
-      <c r="I6" s="12">
+        <v>2</v>
+      </c>
+      <c r="I6" s="1">
         <v>0.11</v>
       </c>
-      <c r="J6" s="11">
+      <c r="J6">
         <f t="shared" si="0"/>
-        <v>0.11</v>
-      </c>
-      <c r="K6" s="12">
+        <v>0.22</v>
+      </c>
+      <c r="K6" s="1">
         <v>100</v>
       </c>
-      <c r="L6" s="12"/>
-      <c r="M6" s="12">
+      <c r="M6" s="1">
         <v>0</v>
       </c>
     </row>
     <row r="7" spans="1:14" s="1" customFormat="1" ht="12.5" x14ac:dyDescent="0.25">
       <c r="A7" s="1" t="s">
-        <v>29</v>
+        <v>26</v>
       </c>
       <c r="B7" s="1" t="s">
-        <v>30</v>
+        <v>27</v>
       </c>
       <c r="C7" s="6" t="s">
-        <v>31</v>
+        <v>28</v>
       </c>
       <c r="E7" s="1" t="s">
         <v>4</v>
       </c>
       <c r="F7" s="1" t="s">
-        <v>106</v>
+        <v>103</v>
       </c>
       <c r="G7" s="6" t="s">
-        <v>32</v>
+        <v>29</v>
       </c>
       <c r="H7" s="1">
         <v>42</v>
       </c>
-      <c r="I7" s="12">
+      <c r="I7" s="1">
         <v>7.0000000000000007E-2</v>
       </c>
-      <c r="J7" s="11">
+      <c r="J7">
         <f t="shared" si="0"/>
         <v>2.9400000000000004</v>
       </c>
-      <c r="K7" s="12"/>
-      <c r="L7" s="12"/>
-      <c r="M7" s="12"/>
     </row>
     <row r="8" spans="1:14" s="1" customFormat="1" ht="12.5" x14ac:dyDescent="0.25">
       <c r="A8" s="1" t="s">
-        <v>95</v>
+        <v>92</v>
       </c>
       <c r="B8" s="1" t="s">
-        <v>96</v>
+        <v>93</v>
       </c>
       <c r="C8" s="6"/>
       <c r="D8" s="1" t="s">
-        <v>98</v>
+        <v>95</v>
       </c>
       <c r="E8" s="1" t="s">
         <v>2</v>
       </c>
       <c r="F8" s="1" t="s">
-        <v>99</v>
+        <v>96</v>
       </c>
       <c r="G8" s="6" t="s">
-        <v>97</v>
+        <v>94</v>
       </c>
       <c r="H8" s="1">
         <v>0</v>
       </c>
-      <c r="I8" s="12">
+      <c r="I8" s="1">
         <v>0.38300000000000001</v>
       </c>
-      <c r="J8" s="11">
+      <c r="J8">
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
-      <c r="K8" s="12"/>
-      <c r="L8" s="12"/>
-      <c r="M8" s="12"/>
       <c r="N8" s="1" t="s">
-        <v>101</v>
+        <v>98</v>
       </c>
     </row>
     <row r="9" spans="1:14" s="1" customFormat="1" ht="12.5" x14ac:dyDescent="0.25">
       <c r="C9" s="6"/>
       <c r="G9" s="6"/>
-      <c r="I9" s="12"/>
-      <c r="J9" s="11"/>
-      <c r="K9" s="12"/>
-      <c r="L9" s="12"/>
-      <c r="M9" s="12"/>
+      <c r="J9"/>
     </row>
     <row r="10" spans="1:14" s="1" customFormat="1" ht="12.5" x14ac:dyDescent="0.25">
       <c r="A10" s="1" t="s">
         <v>12</v>
       </c>
       <c r="B10" s="1" t="s">
-        <v>33</v>
+        <v>30</v>
       </c>
       <c r="C10" s="6" t="s">
-        <v>34</v>
+        <v>31</v>
       </c>
       <c r="E10" s="1" t="s">
         <v>4</v>
       </c>
       <c r="G10" s="10" t="s">
-        <v>35</v>
+        <v>32</v>
       </c>
       <c r="H10" s="1">
         <v>1</v>
       </c>
-      <c r="I10" s="15">
+      <c r="I10" s="13">
         <v>0.08</v>
       </c>
-      <c r="J10" s="11">
+      <c r="J10">
         <v>0.1</v>
       </c>
-      <c r="K10" s="12">
-        <v>0</v>
-      </c>
-      <c r="L10" s="12">
-        <v>0</v>
-      </c>
-      <c r="M10" s="12"/>
+      <c r="K10" s="1">
+        <v>0</v>
+      </c>
+      <c r="L10" s="1">
+        <v>0</v>
+      </c>
     </row>
     <row r="11" spans="1:14" s="1" customFormat="1" ht="12.5" x14ac:dyDescent="0.25">
       <c r="A11" s="1" t="s">
         <v>13</v>
       </c>
       <c r="B11" s="1" t="s">
-        <v>36</v>
+        <v>33</v>
       </c>
       <c r="C11" s="6" t="s">
-        <v>37</v>
+        <v>34</v>
       </c>
       <c r="E11" s="1" t="s">
         <v>4</v>
       </c>
       <c r="F11" s="1" t="s">
-        <v>82</v>
-      </c>
-      <c r="G11" s="19" t="s">
-        <v>91</v>
+        <v>79</v>
+      </c>
+      <c r="G11" s="17" t="s">
+        <v>88</v>
       </c>
       <c r="H11" s="1">
         <v>1</v>
       </c>
-      <c r="I11" s="12">
+      <c r="I11" s="1">
         <v>0.19</v>
       </c>
-      <c r="J11" s="11">
+      <c r="J11">
         <v>0.2</v>
       </c>
-      <c r="K11" s="12">
-        <v>0</v>
-      </c>
-      <c r="L11" s="12">
-        <v>0</v>
-      </c>
-      <c r="M11" s="12"/>
+      <c r="K11" s="1">
+        <v>0</v>
+      </c>
+      <c r="L11" s="1">
+        <v>0</v>
+      </c>
     </row>
     <row r="12" spans="1:14" s="1" customFormat="1" ht="12.5" x14ac:dyDescent="0.25">
+      <c r="A12" s="1" t="s">
+        <v>107</v>
+      </c>
+      <c r="B12" s="1" t="s">
+        <v>108</v>
+      </c>
       <c r="C12" s="6"/>
-      <c r="G12" s="6"/>
-      <c r="I12" s="12"/>
-      <c r="J12" s="11"/>
-      <c r="K12" s="12"/>
-      <c r="L12" s="12"/>
-      <c r="M12" s="12"/>
+      <c r="G12" s="17"/>
+      <c r="J12"/>
+      <c r="N12" s="1" t="s">
+        <v>109</v>
+      </c>
     </row>
     <row r="13" spans="1:14" s="1" customFormat="1" ht="12.5" x14ac:dyDescent="0.25">
       <c r="A13" s="1" t="s">
-        <v>38</v>
+        <v>110</v>
       </c>
       <c r="B13" s="1" t="s">
-        <v>39</v>
-      </c>
-      <c r="C13" s="6" t="s">
+        <v>111</v>
+      </c>
+      <c r="C13" s="6"/>
+      <c r="G13" s="17"/>
+      <c r="J13"/>
+      <c r="N13" s="1" t="s">
+        <v>109</v>
+      </c>
+    </row>
+    <row r="14" spans="1:14" s="1" customFormat="1" ht="12.5" x14ac:dyDescent="0.25">
+      <c r="D14" s="6"/>
+      <c r="H14" s="6"/>
+      <c r="K14"/>
+    </row>
+    <row r="15" spans="1:14" s="1" customFormat="1" ht="12.5" x14ac:dyDescent="0.25">
+      <c r="A15" s="1" t="s">
+        <v>35</v>
+      </c>
+      <c r="B15" s="1" t="s">
+        <v>36</v>
+      </c>
+      <c r="C15" s="6" t="s">
         <v>9</v>
       </c>
-      <c r="G13" s="6" t="s">
-        <v>22</v>
-      </c>
-      <c r="H13" s="1">
+      <c r="G15" s="6" t="s">
+        <v>21</v>
+      </c>
+      <c r="H15" s="1">
         <v>2</v>
       </c>
-      <c r="I13" s="12">
+      <c r="I15" s="1">
         <v>1E-3</v>
       </c>
-      <c r="J13" s="11">
+      <c r="J15">
         <f t="shared" si="0"/>
         <v>2E-3</v>
       </c>
-      <c r="K13" s="12">
-        <v>0</v>
-      </c>
-      <c r="L13" s="12">
-        <v>0</v>
-      </c>
-      <c r="M13" s="12">
+      <c r="K15" s="1">
+        <v>0</v>
+      </c>
+      <c r="L15" s="1">
+        <v>0</v>
+      </c>
+      <c r="M15" s="1">
         <v>5000</v>
       </c>
     </row>
-    <row r="14" spans="1:14" s="1" customFormat="1" ht="12.5" x14ac:dyDescent="0.25">
-      <c r="A14" s="1" t="s">
-        <v>40</v>
-      </c>
-      <c r="B14" s="1" t="s">
-        <v>41</v>
-      </c>
-      <c r="C14" s="6" t="s">
+    <row r="16" spans="1:14" s="1" customFormat="1" ht="12.5" x14ac:dyDescent="0.25">
+      <c r="A16" s="1" t="s">
+        <v>37</v>
+      </c>
+      <c r="B16" s="1" t="s">
+        <v>38</v>
+      </c>
+      <c r="C16" s="6" t="s">
         <v>9</v>
       </c>
-      <c r="G14" s="6" t="s">
-        <v>22</v>
-      </c>
-      <c r="H14" s="1">
+      <c r="G16" s="6" t="s">
+        <v>21</v>
+      </c>
+      <c r="H16" s="1">
         <v>2</v>
       </c>
-      <c r="I14" s="12">
+      <c r="I16" s="1">
         <v>1E-3</v>
       </c>
-      <c r="J14" s="11">
+      <c r="J16">
         <f t="shared" si="0"/>
         <v>2E-3</v>
       </c>
-      <c r="K14" s="12">
-        <v>0</v>
-      </c>
-      <c r="L14" s="12">
-        <v>0</v>
-      </c>
-      <c r="M14" s="12">
+      <c r="K16" s="1">
+        <v>0</v>
+      </c>
+      <c r="L16" s="1">
+        <v>0</v>
+      </c>
+      <c r="M16" s="1">
         <v>5000</v>
       </c>
     </row>
-    <row r="15" spans="1:14" s="1" customFormat="1" ht="12.5" x14ac:dyDescent="0.25">
-      <c r="A15" s="1" t="s">
-        <v>42</v>
-      </c>
-      <c r="B15" s="1" t="s">
-        <v>43</v>
-      </c>
-      <c r="C15" s="6" t="s">
+    <row r="17" spans="1:13" s="1" customFormat="1" ht="12.5" x14ac:dyDescent="0.25">
+      <c r="A17" s="1" t="s">
+        <v>39</v>
+      </c>
+      <c r="B17" s="1" t="s">
+        <v>40</v>
+      </c>
+      <c r="C17" s="6" t="s">
         <v>9</v>
       </c>
-      <c r="G15" s="6" t="s">
-        <v>22</v>
-      </c>
-      <c r="H15" s="1">
+      <c r="G17" s="6" t="s">
+        <v>21</v>
+      </c>
+      <c r="H17" s="1">
         <v>2</v>
       </c>
-      <c r="I15" s="12">
+      <c r="I17" s="1">
         <v>1E-3</v>
       </c>
-      <c r="J15" s="11">
+      <c r="J17">
         <f t="shared" si="0"/>
         <v>2E-3</v>
       </c>
-      <c r="K15" s="12"/>
-      <c r="L15" s="12">
+      <c r="L17" s="1">
         <v>5000</v>
       </c>
-      <c r="M15" s="12"/>
-    </row>
-    <row r="16" spans="1:14" s="1" customFormat="1" ht="12.5" x14ac:dyDescent="0.25">
-      <c r="A16" s="1" t="s">
-        <v>44</v>
-      </c>
-      <c r="B16" s="1" t="s">
-        <v>45</v>
-      </c>
-      <c r="C16" s="6" t="s">
+    </row>
+    <row r="18" spans="1:13" s="1" customFormat="1" ht="12.5" x14ac:dyDescent="0.25">
+      <c r="A18" s="1" t="s">
+        <v>41</v>
+      </c>
+      <c r="B18" s="1" t="s">
+        <v>42</v>
+      </c>
+      <c r="C18" s="6" t="s">
         <v>9</v>
       </c>
-      <c r="G16" s="6" t="s">
-        <v>22</v>
-      </c>
-      <c r="H16" s="1">
+      <c r="G18" s="6" t="s">
+        <v>21</v>
+      </c>
+      <c r="H18" s="1">
         <v>2</v>
       </c>
-      <c r="I16" s="12">
+      <c r="I18" s="1">
         <v>1E-3</v>
       </c>
-      <c r="J16" s="11">
+      <c r="J18">
         <f t="shared" si="0"/>
         <v>2E-3</v>
       </c>
-      <c r="K16" s="12"/>
-      <c r="L16" s="12">
+      <c r="L18" s="1">
         <v>5000</v>
       </c>
-      <c r="M16" s="12"/>
-    </row>
-    <row r="17" spans="1:15" s="1" customFormat="1" ht="12.5" x14ac:dyDescent="0.25">
-      <c r="A17" s="1" t="s">
-        <v>46</v>
-      </c>
-      <c r="B17" s="1" t="s">
+    </row>
+    <row r="19" spans="1:13" s="1" customFormat="1" ht="12.5" x14ac:dyDescent="0.25">
+      <c r="A19" s="1" t="s">
+        <v>43</v>
+      </c>
+      <c r="B19" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="C17" s="6" t="s">
+      <c r="C19" s="6" t="s">
         <v>9</v>
       </c>
-      <c r="G17" s="6" t="s">
-        <v>22</v>
-      </c>
-      <c r="H17" s="1">
+      <c r="G19" s="6" t="s">
+        <v>21</v>
+      </c>
+      <c r="H19" s="1">
         <v>1</v>
       </c>
-      <c r="I17" s="12">
+      <c r="I19" s="1">
         <v>1E-3</v>
       </c>
-      <c r="J17" s="11">
+      <c r="J19">
         <f t="shared" si="0"/>
         <v>1E-3</v>
       </c>
-      <c r="K17" s="12">
-        <v>0</v>
-      </c>
-      <c r="L17" s="12">
-        <v>0</v>
-      </c>
-      <c r="M17" s="12">
+      <c r="K19" s="1">
+        <v>0</v>
+      </c>
+      <c r="L19" s="1">
+        <v>0</v>
+      </c>
+      <c r="M19" s="1">
         <v>5000</v>
       </c>
     </row>
-    <row r="18" spans="1:15" s="1" customFormat="1" ht="12.5" x14ac:dyDescent="0.25">
-      <c r="C18" s="6"/>
-      <c r="G18" s="6"/>
-      <c r="I18" s="12"/>
-      <c r="J18" s="11"/>
-      <c r="K18" s="12"/>
-      <c r="L18" s="12"/>
-      <c r="M18" s="12"/>
-    </row>
-    <row r="19" spans="1:15" s="1" customFormat="1" ht="12.5" x14ac:dyDescent="0.25">
-      <c r="A19" s="1" t="s">
+    <row r="20" spans="1:13" s="1" customFormat="1" ht="12.5" x14ac:dyDescent="0.25">
+      <c r="C20" s="6"/>
+      <c r="G20" s="6"/>
+      <c r="J20"/>
+    </row>
+    <row r="21" spans="1:13" s="1" customFormat="1" ht="12.5" x14ac:dyDescent="0.25">
+      <c r="A21" s="1" t="s">
         <v>14</v>
       </c>
-      <c r="B19" s="1" t="s">
-        <v>47</v>
-      </c>
-      <c r="C19" s="6" t="s">
-        <v>48</v>
-      </c>
-      <c r="D19" s="1" t="s">
-        <v>85</v>
-      </c>
-      <c r="E19" s="1" t="s">
+      <c r="B21" s="1" t="s">
+        <v>44</v>
+      </c>
+      <c r="C21" s="6" t="s">
+        <v>45</v>
+      </c>
+      <c r="D21" s="1" t="s">
+        <v>82</v>
+      </c>
+      <c r="E21" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="F19" s="1" t="s">
-        <v>86</v>
-      </c>
-      <c r="G19" s="6" t="s">
-        <v>22</v>
-      </c>
-      <c r="H19" s="1">
+      <c r="F21" s="1" t="s">
+        <v>83</v>
+      </c>
+      <c r="G21" s="6" t="s">
+        <v>21</v>
+      </c>
+      <c r="H21" s="1">
         <v>1</v>
       </c>
-      <c r="I19" s="12">
+      <c r="I21" s="1">
         <v>0.214</v>
       </c>
-      <c r="J19" s="11">
+      <c r="J21">
         <f t="shared" si="0"/>
         <v>0.214</v>
       </c>
-      <c r="K19" s="12"/>
-      <c r="L19" s="12">
+      <c r="L21" s="1">
         <v>150</v>
       </c>
-      <c r="M19" s="12"/>
-    </row>
-    <row r="20" spans="1:15" s="1" customFormat="1" ht="12.5" x14ac:dyDescent="0.25">
-      <c r="A20" s="1" t="s">
+    </row>
+    <row r="22" spans="1:13" s="1" customFormat="1" ht="12.5" x14ac:dyDescent="0.25">
+      <c r="A22" s="1" t="s">
         <v>15</v>
       </c>
-      <c r="B20" s="1" t="s">
-        <v>49</v>
-      </c>
-      <c r="C20" s="6" t="s">
-        <v>50</v>
-      </c>
-      <c r="D20" s="1" t="s">
+      <c r="B22" s="1" t="s">
+        <v>46</v>
+      </c>
+      <c r="C22" s="6" t="s">
+        <v>47</v>
+      </c>
+      <c r="D22" s="1" t="s">
         <v>11</v>
       </c>
-      <c r="E20" s="1" t="s">
+      <c r="E22" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="F20" s="1" t="s">
+      <c r="F22" s="1" t="s">
         <v>10</v>
       </c>
-      <c r="G20" s="10" t="s">
-        <v>84</v>
-      </c>
-      <c r="H20" s="1">
+      <c r="G22" s="10" t="s">
+        <v>81</v>
+      </c>
+      <c r="H22" s="1">
         <v>1</v>
       </c>
-      <c r="I20" s="15">
+      <c r="I22" s="13">
         <v>0.46300000000000002</v>
       </c>
-      <c r="J20" s="11">
+      <c r="J22">
         <f t="shared" si="0"/>
         <v>0.46300000000000002</v>
       </c>
-      <c r="K20" s="12"/>
-      <c r="L20" s="12">
+      <c r="L22" s="1">
         <v>150</v>
       </c>
-      <c r="M20" s="12"/>
-    </row>
-    <row r="21" spans="1:15" s="1" customFormat="1" ht="12.5" x14ac:dyDescent="0.25">
-      <c r="C21" s="6"/>
-      <c r="G21" s="10"/>
-      <c r="I21" s="13"/>
-      <c r="J21" s="11"/>
-      <c r="K21" s="12"/>
-      <c r="L21" s="12"/>
-      <c r="M21" s="12"/>
-    </row>
-    <row r="22" spans="1:15" s="1" customFormat="1" ht="12.5" x14ac:dyDescent="0.25">
-      <c r="A22" s="1" t="s">
-        <v>51</v>
-      </c>
-      <c r="B22" s="1" t="s">
-        <v>52</v>
-      </c>
-      <c r="C22" s="6" t="s">
-        <v>53</v>
-      </c>
-      <c r="D22" s="1" t="s">
-        <v>83</v>
-      </c>
-      <c r="G22" s="10" t="s">
-        <v>22</v>
-      </c>
-      <c r="H22" s="1">
-        <v>1</v>
-      </c>
-      <c r="I22" s="13"/>
-      <c r="J22" s="11">
-        <f t="shared" si="0"/>
-        <v>0</v>
-      </c>
-      <c r="K22" s="12"/>
-      <c r="L22" s="12"/>
-      <c r="M22" s="12"/>
-    </row>
-    <row r="23" spans="1:15" s="1" customFormat="1" ht="12.5" x14ac:dyDescent="0.25">
+    </row>
+    <row r="23" spans="1:13" s="1" customFormat="1" ht="12.5" x14ac:dyDescent="0.25">
       <c r="A23" s="1" t="s">
-        <v>54</v>
+        <v>112</v>
       </c>
       <c r="B23" s="1" t="s">
-        <v>55</v>
-      </c>
-      <c r="C23" s="6" t="s">
-        <v>53</v>
+        <v>114</v>
+      </c>
+      <c r="C23" s="1" t="s">
+        <v>113</v>
       </c>
       <c r="D23" s="1" t="s">
-        <v>83</v>
-      </c>
-      <c r="G23" s="6" t="s">
-        <v>22</v>
+        <v>113</v>
+      </c>
+      <c r="E23" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="F23" s="1" t="s">
+        <v>115</v>
+      </c>
+      <c r="G23" s="10" t="s">
+        <v>116</v>
       </c>
       <c r="H23" s="1">
         <v>1</v>
       </c>
-      <c r="I23" s="12"/>
-      <c r="J23" s="11">
+      <c r="I23" s="13">
+        <v>2.02</v>
+      </c>
+      <c r="J23">
         <f t="shared" si="0"/>
-        <v>0</v>
-      </c>
-      <c r="K23" s="12"/>
-      <c r="L23" s="12"/>
-      <c r="M23" s="12"/>
-    </row>
-    <row r="24" spans="1:15" s="1" customFormat="1" ht="12.5" x14ac:dyDescent="0.25">
-      <c r="A24" s="1" t="s">
-        <v>56</v>
-      </c>
-      <c r="B24" s="1" t="s">
-        <v>57</v>
-      </c>
-      <c r="C24" s="6" t="s">
-        <v>53</v>
-      </c>
-      <c r="D24" s="1" t="s">
-        <v>83</v>
-      </c>
-      <c r="G24" s="6" t="s">
-        <v>22</v>
-      </c>
-      <c r="H24" s="1">
-        <v>1</v>
-      </c>
-      <c r="I24" s="12"/>
-      <c r="J24" s="11">
-        <f t="shared" si="0"/>
-        <v>0</v>
-      </c>
-      <c r="K24" s="12"/>
-      <c r="L24" s="12"/>
-      <c r="M24" s="12"/>
-    </row>
-    <row r="25" spans="1:15" s="1" customFormat="1" ht="12.5" x14ac:dyDescent="0.25">
+        <v>2.02</v>
+      </c>
+      <c r="K23" s="1">
+        <v>0</v>
+      </c>
+      <c r="L23" s="1">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="24" spans="1:13" s="1" customFormat="1" ht="12.5" x14ac:dyDescent="0.25">
+      <c r="C24" s="6"/>
+      <c r="G24" s="10"/>
+      <c r="I24" s="11"/>
+      <c r="J24"/>
+    </row>
+    <row r="25" spans="1:13" s="1" customFormat="1" ht="12.5" x14ac:dyDescent="0.25">
       <c r="A25" s="1" t="s">
-        <v>58</v>
+        <v>48</v>
       </c>
       <c r="B25" s="1" t="s">
-        <v>59</v>
+        <v>49</v>
       </c>
       <c r="C25" s="6" t="s">
-        <v>53</v>
+        <v>50</v>
       </c>
       <c r="D25" s="1" t="s">
-        <v>83</v>
-      </c>
-      <c r="G25" s="6" t="s">
-        <v>22</v>
+        <v>80</v>
+      </c>
+      <c r="G25" s="10" t="s">
+        <v>21</v>
       </c>
       <c r="H25" s="1">
         <v>1</v>
       </c>
-      <c r="I25" s="12"/>
-      <c r="J25" s="11">
+      <c r="I25" s="11"/>
+      <c r="J25">
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
-      <c r="K25" s="12"/>
-      <c r="L25" s="12"/>
-      <c r="M25" s="12"/>
-    </row>
-    <row r="26" spans="1:15" s="1" customFormat="1" ht="12.5" x14ac:dyDescent="0.25">
-      <c r="C26" s="6"/>
-      <c r="G26" s="6"/>
-      <c r="I26" s="12"/>
-      <c r="J26" s="11"/>
-      <c r="K26" s="12"/>
-      <c r="L26" s="12"/>
-      <c r="M26" s="12"/>
-    </row>
-    <row r="27" spans="1:15" s="1" customFormat="1" ht="12.5" x14ac:dyDescent="0.25">
+    </row>
+    <row r="26" spans="1:13" s="1" customFormat="1" ht="12.5" x14ac:dyDescent="0.25">
+      <c r="A26" s="1" t="s">
+        <v>51</v>
+      </c>
+      <c r="B26" s="1" t="s">
+        <v>52</v>
+      </c>
+      <c r="C26" s="6" t="s">
+        <v>50</v>
+      </c>
+      <c r="D26" s="1" t="s">
+        <v>80</v>
+      </c>
+      <c r="G26" s="6" t="s">
+        <v>21</v>
+      </c>
+      <c r="H26" s="1">
+        <v>1</v>
+      </c>
+      <c r="J26">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="27" spans="1:13" s="1" customFormat="1" ht="12.5" x14ac:dyDescent="0.25">
       <c r="A27" s="1" t="s">
-        <v>6</v>
+        <v>53</v>
       </c>
       <c r="B27" s="1" t="s">
-        <v>60</v>
+        <v>54</v>
       </c>
       <c r="C27" s="6" t="s">
-        <v>61</v>
+        <v>50</v>
       </c>
       <c r="D27" s="1" t="s">
-        <v>60</v>
-      </c>
-      <c r="E27" s="1" t="s">
-        <v>2</v>
-      </c>
-      <c r="F27" s="1" t="s">
-        <v>87</v>
+        <v>80</v>
       </c>
       <c r="G27" s="6" t="s">
-        <v>62</v>
+        <v>21</v>
       </c>
       <c r="H27" s="1">
         <v>1</v>
       </c>
-      <c r="I27" s="12">
+      <c r="J27">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="28" spans="1:13" s="1" customFormat="1" ht="12.5" x14ac:dyDescent="0.25">
+      <c r="A28" s="1" t="s">
+        <v>55</v>
+      </c>
+      <c r="B28" s="1" t="s">
+        <v>56</v>
+      </c>
+      <c r="C28" s="6" t="s">
+        <v>50</v>
+      </c>
+      <c r="D28" s="1" t="s">
+        <v>80</v>
+      </c>
+      <c r="G28" s="6" t="s">
+        <v>21</v>
+      </c>
+      <c r="H28" s="1">
+        <v>1</v>
+      </c>
+      <c r="J28">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="29" spans="1:13" s="1" customFormat="1" ht="12.5" x14ac:dyDescent="0.25">
+      <c r="A29" s="1" t="s">
+        <v>117</v>
+      </c>
+      <c r="B29" s="1" t="s">
+        <v>118</v>
+      </c>
+      <c r="C29" s="6"/>
+      <c r="D29" s="1" t="s">
+        <v>80</v>
+      </c>
+      <c r="G29" s="6"/>
+      <c r="J29"/>
+    </row>
+    <row r="30" spans="1:13" s="1" customFormat="1" ht="12.5" x14ac:dyDescent="0.25">
+      <c r="C30" s="6"/>
+      <c r="G30" s="6"/>
+      <c r="J30"/>
+    </row>
+    <row r="31" spans="1:13" s="1" customFormat="1" ht="12.5" x14ac:dyDescent="0.25">
+      <c r="A31" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="B31" s="1" t="s">
+        <v>57</v>
+      </c>
+      <c r="C31" s="6" t="s">
+        <v>58</v>
+      </c>
+      <c r="D31" s="1" t="s">
+        <v>57</v>
+      </c>
+      <c r="E31" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="F31" s="1" t="s">
+        <v>84</v>
+      </c>
+      <c r="G31" s="6" t="s">
+        <v>59</v>
+      </c>
+      <c r="H31" s="1">
+        <v>1</v>
+      </c>
+      <c r="I31" s="1">
         <v>9.9000000000000005E-2</v>
       </c>
-      <c r="J27" s="11">
+      <c r="J31">
         <f t="shared" si="0"/>
         <v>9.9000000000000005E-2</v>
       </c>
-      <c r="K27" s="12">
-        <v>0</v>
-      </c>
-      <c r="L27" s="12">
-        <v>0</v>
-      </c>
-      <c r="M27" s="12">
+      <c r="K31" s="1">
+        <v>0</v>
+      </c>
+      <c r="L31" s="1">
+        <v>0</v>
+      </c>
+      <c r="M31" s="1">
         <v>3000</v>
       </c>
     </row>
-    <row r="28" spans="1:15" s="1" customFormat="1" ht="12.5" x14ac:dyDescent="0.25">
-      <c r="A28" s="1" t="s">
+    <row r="32" spans="1:13" s="1" customFormat="1" ht="12.5" x14ac:dyDescent="0.25">
+      <c r="A32" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="B28" s="1" t="s">
-        <v>63</v>
-      </c>
-      <c r="C28" s="6" t="s">
-        <v>64</v>
-      </c>
-      <c r="D28" s="1" t="s">
-        <v>80</v>
-      </c>
-      <c r="E28" s="1" t="s">
+      <c r="B32" s="1" t="s">
+        <v>60</v>
+      </c>
+      <c r="C32" s="6" t="s">
+        <v>61</v>
+      </c>
+      <c r="D32" s="1" t="s">
+        <v>77</v>
+      </c>
+      <c r="E32" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="F28" s="1" t="s">
-        <v>81</v>
-      </c>
-      <c r="G28" s="9" t="s">
-        <v>65</v>
-      </c>
-      <c r="H28" s="1">
+      <c r="F32" s="1" t="s">
+        <v>78</v>
+      </c>
+      <c r="G32" s="9" t="s">
+        <v>62</v>
+      </c>
+      <c r="H32" s="1">
         <v>1</v>
       </c>
-      <c r="I28" s="14">
+      <c r="I32" s="12">
         <v>0.8</v>
       </c>
-      <c r="J28" s="11">
+      <c r="J32">
         <f t="shared" si="0"/>
         <v>0.8</v>
       </c>
-      <c r="K28" s="12">
-        <v>0</v>
-      </c>
-      <c r="L28" s="12">
-        <v>0</v>
-      </c>
-      <c r="M28" s="12"/>
-    </row>
-    <row r="29" spans="1:15" s="1" customFormat="1" ht="12.5" x14ac:dyDescent="0.25">
-      <c r="A29" s="1" t="s">
+      <c r="K32" s="1">
+        <v>0</v>
+      </c>
+      <c r="L32" s="1">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="33" spans="1:15" s="1" customFormat="1" ht="12.5" x14ac:dyDescent="0.25">
+      <c r="A33" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="B29" s="1" t="s">
-        <v>66</v>
-      </c>
-      <c r="C29" s="6" t="s">
-        <v>67</v>
-      </c>
-      <c r="D29" s="1" t="s">
-        <v>88</v>
-      </c>
-      <c r="E29" s="1" t="s">
+      <c r="B33" s="1" t="s">
+        <v>63</v>
+      </c>
+      <c r="C33" s="6" t="s">
+        <v>64</v>
+      </c>
+      <c r="D33" s="1" t="s">
+        <v>85</v>
+      </c>
+      <c r="E33" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="F29" s="1" t="s">
-        <v>89</v>
-      </c>
-      <c r="G29" s="6" t="s">
-        <v>90</v>
-      </c>
-      <c r="H29" s="1">
+      <c r="F33" s="1" t="s">
+        <v>86</v>
+      </c>
+      <c r="G33" s="6" t="s">
+        <v>87</v>
+      </c>
+      <c r="H33" s="1">
         <v>1</v>
       </c>
-      <c r="I29" s="15">
+      <c r="I33" s="13">
         <v>0.48099999999999998</v>
       </c>
-      <c r="J29" s="11">
+      <c r="J33">
         <f t="shared" si="0"/>
         <v>0.48099999999999998</v>
       </c>
-      <c r="K29" s="12"/>
-      <c r="L29" s="12">
+      <c r="L33" s="1">
         <v>150</v>
       </c>
-      <c r="M29" s="12"/>
-    </row>
-    <row r="30" spans="1:15" s="1" customFormat="1" ht="12.5" x14ac:dyDescent="0.25">
-      <c r="C30" s="6"/>
-      <c r="G30" s="6"/>
-      <c r="I30" s="13"/>
-      <c r="J30" s="11"/>
-      <c r="K30" s="12"/>
-      <c r="L30" s="12"/>
-      <c r="M30" s="12"/>
-    </row>
-    <row r="31" spans="1:15" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A31" t="s">
+    </row>
+    <row r="34" spans="1:15" s="1" customFormat="1" ht="12.5" x14ac:dyDescent="0.25">
+      <c r="A34" s="1" t="s">
+        <v>119</v>
+      </c>
+      <c r="B34" s="1" t="s">
+        <v>120</v>
+      </c>
+      <c r="C34" s="6" t="s">
+        <v>121</v>
+      </c>
+      <c r="D34" s="1" t="s">
+        <v>120</v>
+      </c>
+      <c r="E34" s="1" t="s">
+        <v>122</v>
+      </c>
+      <c r="F34" s="1" t="s">
+        <v>123</v>
+      </c>
+      <c r="G34" s="6" t="s">
+        <v>124</v>
+      </c>
+      <c r="H34" s="1">
+        <v>1</v>
+      </c>
+      <c r="I34" s="13">
+        <v>0.58679999999999999</v>
+      </c>
+      <c r="J34">
+        <f t="shared" si="0"/>
+        <v>0.58679999999999999</v>
+      </c>
+      <c r="K34" s="1">
+        <v>0</v>
+      </c>
+      <c r="L34" s="1">
+        <v>150</v>
+      </c>
+    </row>
+    <row r="35" spans="1:15" s="1" customFormat="1" ht="12.5" x14ac:dyDescent="0.25">
+      <c r="A35" s="1" t="s">
+        <v>125</v>
+      </c>
+      <c r="B35" s="1" t="s">
+        <v>126</v>
+      </c>
+      <c r="C35" s="6" t="s">
+        <v>127</v>
+      </c>
+      <c r="D35" s="1" t="s">
+        <v>126</v>
+      </c>
+      <c r="E35" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="G35" s="6"/>
+      <c r="H35" s="1">
+        <v>1</v>
+      </c>
+      <c r="I35" s="13">
+        <f>5.42/5</f>
+        <v>1.0840000000000001</v>
+      </c>
+      <c r="J35">
+        <f t="shared" si="0"/>
+        <v>1.0840000000000001</v>
+      </c>
+      <c r="K35" s="1">
+        <v>0</v>
+      </c>
+      <c r="L35" s="1">
+        <v>175</v>
+      </c>
+    </row>
+    <row r="36" spans="1:15" s="1" customFormat="1" ht="12.5" x14ac:dyDescent="0.25">
+      <c r="C36" s="6"/>
+      <c r="G36" s="6"/>
+      <c r="I36" s="11"/>
+      <c r="J36"/>
+    </row>
+    <row r="37" spans="1:15" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A37" t="s">
+        <v>65</v>
+      </c>
+      <c r="B37" t="s">
+        <v>66</v>
+      </c>
+      <c r="C37" s="5" t="s">
+        <v>67</v>
+      </c>
+      <c r="D37" s="3" t="s">
+        <v>80</v>
+      </c>
+      <c r="H37">
+        <v>1</v>
+      </c>
+      <c r="J37">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+      <c r="O37" s="1"/>
+    </row>
+    <row r="38" spans="1:15" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="D38" s="3"/>
+      <c r="J38"/>
+      <c r="O38" s="1"/>
+    </row>
+    <row r="39" spans="1:15" s="1" customFormat="1" ht="12.5" x14ac:dyDescent="0.25">
+      <c r="A39" s="1" t="s">
         <v>68</v>
       </c>
-      <c r="B31" t="s">
+      <c r="B39" s="1" t="s">
         <v>69</v>
       </c>
-      <c r="C31" s="5" t="s">
+      <c r="C39" s="6" t="s">
         <v>70</v>
       </c>
-      <c r="D31" s="3" t="s">
-        <v>83</v>
-      </c>
-      <c r="H31">
+      <c r="D39" s="1" t="s">
+        <v>89</v>
+      </c>
+      <c r="E39" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="F39" s="1" t="s">
+        <v>90</v>
+      </c>
+      <c r="G39" s="6" t="s">
+        <v>91</v>
+      </c>
+      <c r="H39" s="1">
         <v>1</v>
       </c>
-      <c r="I31" s="11"/>
-      <c r="J31" s="11">
-        <f t="shared" si="0"/>
-        <v>0</v>
-      </c>
-      <c r="K31" s="11"/>
-      <c r="L31" s="11"/>
-      <c r="M31" s="11"/>
-      <c r="O31" s="1"/>
-    </row>
-    <row r="32" spans="1:15" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="D32" s="3"/>
-      <c r="I32" s="11"/>
-      <c r="J32" s="11"/>
-      <c r="K32" s="11"/>
-      <c r="L32" s="11"/>
-      <c r="M32" s="11"/>
-      <c r="O32" s="1"/>
-    </row>
-    <row r="33" spans="1:13" s="1" customFormat="1" ht="12.5" x14ac:dyDescent="0.25">
-      <c r="A33" s="1" t="s">
-        <v>71</v>
-      </c>
-      <c r="B33" s="1" t="s">
-        <v>72</v>
-      </c>
-      <c r="C33" s="6" t="s">
-        <v>73</v>
-      </c>
-      <c r="D33" s="1" t="s">
-        <v>92</v>
-      </c>
-      <c r="E33" s="1" t="s">
-        <v>2</v>
-      </c>
-      <c r="F33" s="1" t="s">
-        <v>93</v>
-      </c>
-      <c r="G33" s="6" t="s">
-        <v>94</v>
-      </c>
-      <c r="H33" s="1">
-        <v>1</v>
-      </c>
-      <c r="I33" s="12">
+      <c r="I39" s="1">
         <v>0.40899999999999997</v>
       </c>
-      <c r="J33" s="11">
+      <c r="J39">
         <f t="shared" si="0"/>
         <v>0.40899999999999997</v>
       </c>
-      <c r="K33" s="12"/>
-      <c r="L33" s="12">
+      <c r="L39" s="1">
         <v>150</v>
       </c>
-      <c r="M33" s="12"/>
-    </row>
-    <row r="34" spans="1:13" s="1" customFormat="1" ht="12.5" x14ac:dyDescent="0.25">
-      <c r="C34" s="6"/>
-      <c r="G34" s="6"/>
-      <c r="I34" s="12"/>
-      <c r="J34" s="11"/>
-      <c r="K34" s="12"/>
-      <c r="L34" s="12"/>
-      <c r="M34" s="12"/>
-    </row>
-    <row r="35" spans="1:13" s="1" customFormat="1" ht="12.5" x14ac:dyDescent="0.25">
-      <c r="C35" s="6"/>
-      <c r="G35" s="6"/>
-      <c r="I35" s="12"/>
-      <c r="J35" s="11"/>
-      <c r="K35" s="12"/>
-      <c r="L35" s="12"/>
-      <c r="M35" s="12"/>
-    </row>
-    <row r="36" spans="1:13" s="1" customFormat="1" ht="13" x14ac:dyDescent="0.3">
-      <c r="A36" s="2" t="s">
-        <v>103</v>
-      </c>
-      <c r="B36" s="1" t="s">
-        <v>104</v>
-      </c>
-      <c r="C36" s="6"/>
-      <c r="E36" s="1" t="s">
+    </row>
+    <row r="40" spans="1:15" s="1" customFormat="1" ht="12.5" x14ac:dyDescent="0.25">
+      <c r="C40" s="6"/>
+      <c r="G40" s="6"/>
+      <c r="J40"/>
+    </row>
+    <row r="41" spans="1:15" s="1" customFormat="1" ht="12.5" x14ac:dyDescent="0.25">
+      <c r="C41" s="6"/>
+      <c r="G41" s="6"/>
+      <c r="J41"/>
+    </row>
+    <row r="42" spans="1:15" s="1" customFormat="1" ht="13" x14ac:dyDescent="0.3">
+      <c r="A42" s="2" t="s">
+        <v>100</v>
+      </c>
+      <c r="B42" s="1" t="s">
+        <v>101</v>
+      </c>
+      <c r="C42" s="6"/>
+      <c r="E42" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="F36" s="1" t="s">
-        <v>105</v>
-      </c>
-      <c r="G36" s="6"/>
-      <c r="H36" s="1">
+      <c r="F42" s="1" t="s">
+        <v>102</v>
+      </c>
+      <c r="G42" s="6"/>
+      <c r="H42" s="1">
         <v>1</v>
       </c>
-      <c r="I36" s="12">
+      <c r="I42" s="1">
         <f>2.53/5</f>
         <v>0.50600000000000001</v>
       </c>
-      <c r="J36" s="11">
+      <c r="J42">
         <f t="shared" si="0"/>
         <v>0.50600000000000001</v>
       </c>
-      <c r="K36" s="12"/>
-      <c r="L36" s="12">
+      <c r="L42" s="1">
         <v>125</v>
       </c>
-      <c r="M36" s="12"/>
-    </row>
-    <row r="37" spans="1:13" s="1" customFormat="1" ht="13" x14ac:dyDescent="0.3">
-      <c r="A37" s="2"/>
-      <c r="C37" s="6"/>
-      <c r="G37" s="6"/>
-      <c r="I37" s="12"/>
-      <c r="J37" s="12"/>
-      <c r="K37" s="12"/>
-      <c r="L37" s="12"/>
-      <c r="M37" s="12"/>
-    </row>
-    <row r="38" spans="1:13" s="1" customFormat="1" ht="13" x14ac:dyDescent="0.3">
-      <c r="A38" s="2"/>
-      <c r="C38" s="6"/>
-      <c r="G38" s="6"/>
-      <c r="I38" s="12"/>
-      <c r="J38" s="12"/>
-      <c r="K38" s="12"/>
-      <c r="L38" s="12"/>
-      <c r="M38" s="12"/>
-    </row>
-    <row r="39" spans="1:13" s="1" customFormat="1" ht="13" x14ac:dyDescent="0.3">
-      <c r="A39" s="2"/>
-      <c r="C39" s="6"/>
-      <c r="G39" s="6"/>
-      <c r="H39" s="1" t="s">
-        <v>107</v>
-      </c>
-      <c r="I39" s="12"/>
-      <c r="J39" s="12">
-        <f>SUM(J2:J36)</f>
-        <v>6.4029999999999996</v>
-      </c>
-      <c r="K39" s="12"/>
-      <c r="L39" s="12"/>
-      <c r="M39" s="12"/>
-    </row>
-    <row r="40" spans="1:13" s="1" customFormat="1" ht="13" x14ac:dyDescent="0.3">
-      <c r="A40" s="2"/>
-      <c r="C40" s="6"/>
-      <c r="G40" s="6"/>
-      <c r="J40" s="6"/>
-    </row>
-    <row r="41" spans="1:13" s="1" customFormat="1" ht="13" x14ac:dyDescent="0.3">
-      <c r="A41" s="2"/>
-      <c r="C41" s="6"/>
-      <c r="G41" s="6"/>
-      <c r="J41" s="6"/>
-    </row>
-    <row r="42" spans="1:13" s="1" customFormat="1" ht="13" x14ac:dyDescent="0.3">
-      <c r="A42" s="2"/>
-      <c r="C42" s="6"/>
-      <c r="G42" s="6"/>
-      <c r="J42" s="6"/>
-    </row>
-    <row r="43" spans="1:13" s="1" customFormat="1" ht="13" x14ac:dyDescent="0.3">
+    </row>
+    <row r="43" spans="1:15" s="1" customFormat="1" ht="13" x14ac:dyDescent="0.3">
       <c r="A43" s="2"/>
+      <c r="B43" s="1" t="s">
+        <v>129</v>
+      </c>
       <c r="C43" s="6"/>
       <c r="G43" s="6"/>
-      <c r="J43" s="6"/>
-    </row>
-    <row r="44" spans="1:13" s="1" customFormat="1" ht="13" x14ac:dyDescent="0.3">
+      <c r="H43" s="1">
+        <v>1</v>
+      </c>
+      <c r="I43" s="1">
+        <v>2.1749999999999998</v>
+      </c>
+      <c r="J43">
+        <f t="shared" si="0"/>
+        <v>2.1749999999999998</v>
+      </c>
+      <c r="L43" s="1">
+        <v>200</v>
+      </c>
+    </row>
+    <row r="44" spans="1:15" s="1" customFormat="1" ht="13" x14ac:dyDescent="0.3">
       <c r="A44" s="2"/>
+      <c r="B44" s="1" t="s">
+        <v>130</v>
+      </c>
       <c r="C44" s="6"/>
+      <c r="E44" s="1" t="s">
+        <v>131</v>
+      </c>
       <c r="G44" s="6"/>
-      <c r="J44" s="6"/>
-    </row>
-    <row r="45" spans="1:13" s="1" customFormat="1" ht="12.5" x14ac:dyDescent="0.25">
+      <c r="H44" s="1">
+        <v>3</v>
+      </c>
+      <c r="I44" s="1">
+        <v>0.15</v>
+      </c>
+      <c r="J44">
+        <f t="shared" si="0"/>
+        <v>0.44999999999999996</v>
+      </c>
+      <c r="L44" s="1">
+        <v>300</v>
+      </c>
+    </row>
+    <row r="45" spans="1:15" s="1" customFormat="1" ht="13" x14ac:dyDescent="0.3">
+      <c r="A45" s="2"/>
       <c r="C45" s="6"/>
       <c r="G45" s="6"/>
-      <c r="J45" s="6"/>
-    </row>
-    <row r="46" spans="1:13" s="4" customFormat="1" ht="13" x14ac:dyDescent="0.3">
-      <c r="C46" s="7"/>
-      <c r="G46" s="7"/>
-      <c r="J46" s="7"/>
-    </row>
-    <row r="47" spans="1:13" s="1" customFormat="1" ht="12.5" x14ac:dyDescent="0.25">
+    </row>
+    <row r="46" spans="1:15" s="1" customFormat="1" ht="13" x14ac:dyDescent="0.3">
+      <c r="A46" s="2"/>
+      <c r="C46" s="6"/>
+      <c r="G46" s="6"/>
+      <c r="H46" s="1" t="s">
+        <v>128</v>
+      </c>
+      <c r="J46" s="1">
+        <f>SUM(J2:J45)</f>
+        <v>12.836799999999997</v>
+      </c>
+    </row>
+    <row r="47" spans="1:15" s="1" customFormat="1" ht="13" x14ac:dyDescent="0.3">
+      <c r="A47" s="2"/>
       <c r="C47" s="6"/>
       <c r="G47" s="6"/>
       <c r="J47" s="6"/>
     </row>
-    <row r="48" spans="1:13" ht="12.5" x14ac:dyDescent="0.25">
-      <c r="B48" s="1"/>
-      <c r="J48" s="8"/>
-    </row>
-    <row r="49" spans="2:2" ht="12.5" x14ac:dyDescent="0.25">
-      <c r="B49" s="1"/>
-    </row>
-    <row r="50" spans="2:2" ht="12.5" x14ac:dyDescent="0.25"/>
-    <row r="51" spans="2:2" ht="12.5" x14ac:dyDescent="0.25"/>
-    <row r="52" spans="2:2" ht="12.5" x14ac:dyDescent="0.25"/>
-    <row r="53" spans="2:2" ht="12.5" x14ac:dyDescent="0.25"/>
-    <row r="54" spans="2:2" ht="12.5" x14ac:dyDescent="0.25"/>
-    <row r="55" spans="2:2" ht="12.5" x14ac:dyDescent="0.25"/>
-    <row r="56" spans="2:2" ht="12.5" x14ac:dyDescent="0.25"/>
-    <row r="57" spans="2:2" ht="12.5" x14ac:dyDescent="0.25"/>
-    <row r="58" spans="2:2" ht="12.5" x14ac:dyDescent="0.25"/>
-    <row r="59" spans="2:2" ht="12.5" x14ac:dyDescent="0.25"/>
-    <row r="60" spans="2:2" ht="12.5" x14ac:dyDescent="0.25"/>
-    <row r="61" spans="2:2" ht="12.5" x14ac:dyDescent="0.25"/>
-    <row r="62" spans="2:2" ht="12.5" x14ac:dyDescent="0.25"/>
-    <row r="63" spans="2:2" ht="12.5" x14ac:dyDescent="0.25"/>
-    <row r="64" spans="2:2" ht="12.5" x14ac:dyDescent="0.25"/>
+    <row r="48" spans="1:15" s="1" customFormat="1" ht="13" x14ac:dyDescent="0.3">
+      <c r="A48" s="2"/>
+      <c r="C48" s="6"/>
+      <c r="G48" s="6"/>
+      <c r="J48" s="6"/>
+    </row>
+    <row r="49" spans="1:10" s="1" customFormat="1" ht="13" x14ac:dyDescent="0.3">
+      <c r="A49" s="2"/>
+      <c r="C49" s="6"/>
+      <c r="G49" s="6"/>
+      <c r="J49" s="6"/>
+    </row>
+    <row r="50" spans="1:10" s="1" customFormat="1" ht="13" x14ac:dyDescent="0.3">
+      <c r="A50" s="2"/>
+      <c r="C50" s="6"/>
+      <c r="G50" s="6"/>
+      <c r="J50" s="6"/>
+    </row>
+    <row r="51" spans="1:10" s="1" customFormat="1" ht="13" x14ac:dyDescent="0.3">
+      <c r="A51" s="2"/>
+      <c r="C51" s="6"/>
+      <c r="G51" s="6"/>
+      <c r="J51" s="6"/>
+    </row>
+    <row r="52" spans="1:10" s="1" customFormat="1" ht="12.5" x14ac:dyDescent="0.25">
+      <c r="C52" s="6"/>
+      <c r="G52" s="6"/>
+      <c r="J52" s="6"/>
+    </row>
+    <row r="53" spans="1:10" s="4" customFormat="1" ht="13" x14ac:dyDescent="0.3">
+      <c r="C53" s="7"/>
+      <c r="G53" s="7"/>
+      <c r="J53" s="7"/>
+    </row>
+    <row r="54" spans="1:10" s="1" customFormat="1" ht="12.5" x14ac:dyDescent="0.25">
+      <c r="C54" s="6"/>
+      <c r="G54" s="6"/>
+      <c r="J54" s="6"/>
+    </row>
+    <row r="55" spans="1:10" ht="12.5" x14ac:dyDescent="0.25">
+      <c r="B55" s="1"/>
+      <c r="J55" s="8"/>
+    </row>
+    <row r="56" spans="1:10" ht="12.5" x14ac:dyDescent="0.25">
+      <c r="B56" s="1"/>
+    </row>
+    <row r="57" spans="1:10" ht="12.5" x14ac:dyDescent="0.25"/>
+    <row r="58" spans="1:10" ht="12.5" x14ac:dyDescent="0.25"/>
+    <row r="59" spans="1:10" ht="12.5" x14ac:dyDescent="0.25"/>
+    <row r="60" spans="1:10" ht="12.5" x14ac:dyDescent="0.25"/>
+    <row r="61" spans="1:10" ht="12.5" x14ac:dyDescent="0.25"/>
+    <row r="62" spans="1:10" ht="12.5" x14ac:dyDescent="0.25"/>
+    <row r="63" spans="1:10" ht="12.5" x14ac:dyDescent="0.25"/>
+    <row r="64" spans="1:10" ht="12.5" x14ac:dyDescent="0.25"/>
     <row r="65" ht="12.5" x14ac:dyDescent="0.25"/>
     <row r="66" ht="12.5" x14ac:dyDescent="0.25"/>
     <row r="67" ht="12.5" x14ac:dyDescent="0.25"/>
@@ -2759,6 +2920,13 @@
     <row r="979" ht="12.5" x14ac:dyDescent="0.25"/>
     <row r="980" ht="12.5" x14ac:dyDescent="0.25"/>
     <row r="981" ht="12.5" x14ac:dyDescent="0.25"/>
+    <row r="982" ht="12.5" x14ac:dyDescent="0.25"/>
+    <row r="983" ht="12.5" x14ac:dyDescent="0.25"/>
+    <row r="984" ht="12.5" x14ac:dyDescent="0.25"/>
+    <row r="985" ht="12.5" x14ac:dyDescent="0.25"/>
+    <row r="986" ht="12.5" x14ac:dyDescent="0.25"/>
+    <row r="987" ht="12.5" x14ac:dyDescent="0.25"/>
+    <row r="988" ht="12.5" x14ac:dyDescent="0.25"/>
   </sheetData>
   <phoneticPr fontId="8" type="noConversion"/>
   <hyperlinks>

</xml_diff>